<commit_message>
refractor: update data cleaning Jupyter Notebook and data output
</commit_message>
<xml_diff>
--- a/src/data_cleaning/data/cleaned/cleaned_no_header_assignments.xlsx
+++ b/src/data_cleaning/data/cleaned/cleaned_no_header_assignments.xlsx
@@ -14,13 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="74">
-  <si>
-    <t>TAS-001</t>
-  </si>
-  <si>
-    <t>TAS-002</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
   <si>
     <t>TAS-003</t>
   </si>
@@ -28,9 +22,6 @@
     <t>TAS-004</t>
   </si>
   <si>
-    <t>TAS-005</t>
-  </si>
-  <si>
     <t>TAS-006</t>
   </si>
   <si>
@@ -55,129 +46,129 @@
     <t>TAS-013</t>
   </si>
   <si>
+    <t>Jason Teo</t>
+  </si>
+  <si>
+    <t>Sarah Lim</t>
+  </si>
+  <si>
+    <t>David Kwok</t>
+  </si>
+  <si>
+    <t>Nurul Huda</t>
+  </si>
+  <si>
+    <t>Marcus Chan</t>
+  </si>
+  <si>
+    <t>Priya Nair</t>
+  </si>
+  <si>
+    <t>Li Mei</t>
+  </si>
+  <si>
     <t>Ahmad Rizwan</t>
   </si>
   <si>
-    <t>Priya Nair</t>
-  </si>
-  <si>
-    <t>Jason Teo</t>
-  </si>
-  <si>
-    <t>Sarah Lim</t>
-  </si>
-  <si>
-    <t>David Kwok</t>
-  </si>
-  <si>
-    <t>Nurul Huda</t>
-  </si>
-  <si>
-    <t>Marcus Chan</t>
-  </si>
-  <si>
-    <t>Li Mei</t>
+    <t>Muhammad Hafiz</t>
+  </si>
+  <si>
+    <t>Chloe Wong</t>
+  </si>
+  <si>
+    <t>Ethan Ng</t>
+  </si>
+  <si>
+    <t>Aisha Binte Yusof</t>
+  </si>
+  <si>
+    <t>Tan Xiu Ying</t>
+  </si>
+  <si>
+    <t>Darren Foo</t>
+  </si>
+  <si>
+    <t>Raeanne Ong</t>
+  </si>
+  <si>
+    <t>Jordan Tan</t>
   </si>
   <si>
     <t>Lim Wei Jie</t>
   </si>
   <si>
-    <t>Tan Xiu Ying</t>
-  </si>
-  <si>
-    <t>Muhammad Hafiz</t>
-  </si>
-  <si>
-    <t>Chloe Wong</t>
-  </si>
-  <si>
-    <t>Ethan Ng</t>
-  </si>
-  <si>
-    <t>Aisha Binte Yusof</t>
-  </si>
-  <si>
-    <t>Darren Foo</t>
-  </si>
-  <si>
-    <t>Raeanne Ong</t>
-  </si>
-  <si>
-    <t>Jordan Tan</t>
-  </si>
-  <si>
     <t>Mathematics</t>
   </si>
   <si>
+    <t>Science</t>
+  </si>
+  <si>
+    <t>Chemistry</t>
+  </si>
+  <si>
+    <t>Physics</t>
+  </si>
+  <si>
     <t>English</t>
   </si>
   <si>
-    <t>Science</t>
-  </si>
-  <si>
-    <t>Chemistry</t>
-  </si>
-  <si>
-    <t>Physics</t>
-  </si>
-  <si>
     <t>Biology</t>
   </si>
   <si>
+    <t>Secondary 4</t>
+  </si>
+  <si>
+    <t>Primary 6</t>
+  </si>
+  <si>
+    <t>Junior College 1</t>
+  </si>
+  <si>
+    <t>Secondary 2</t>
+  </si>
+  <si>
+    <t>Secondary 1</t>
+  </si>
+  <si>
+    <t>Primary 5</t>
+  </si>
+  <si>
     <t>Secondary 3</t>
   </si>
   <si>
-    <t>Primary 5</t>
-  </si>
-  <si>
-    <t>Secondary 4</t>
-  </si>
-  <si>
-    <t>Primary 6</t>
-  </si>
-  <si>
-    <t>Junior College 1</t>
-  </si>
-  <si>
-    <t>Secondary 2</t>
-  </si>
-  <si>
-    <t>Secondary 1</t>
-  </si>
-  <si>
     <t>Primary 4</t>
   </si>
   <si>
+    <t>2025-02-12</t>
+  </si>
+  <si>
+    <t>2025-03-18</t>
+  </si>
+  <si>
+    <t>2025-04-25</t>
+  </si>
+  <si>
+    <t>2025-06-01</t>
+  </si>
+  <si>
+    <t>2025-07-07</t>
+  </si>
+  <si>
+    <t>2025-03-12</t>
+  </si>
+  <si>
+    <t>2025-08-20</t>
+  </si>
+  <si>
+    <t>2025-09-01</t>
+  </si>
+  <si>
+    <t>2025-10-15</t>
+  </si>
+  <si>
     <t>2025-01-05</t>
   </si>
   <si>
-    <t>2025-03-12</t>
-  </si>
-  <si>
-    <t>2025-02-12</t>
-  </si>
-  <si>
-    <t>2025-03-18</t>
-  </si>
-  <si>
-    <t>2025-04-25</t>
-  </si>
-  <si>
-    <t>2025-06-01</t>
-  </si>
-  <si>
-    <t>2025-07-07</t>
-  </si>
-  <si>
-    <t>2025-08-20</t>
-  </si>
-  <si>
-    <t>2025-09-01</t>
-  </si>
-  <si>
-    <t>2025-10-15</t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
@@ -187,28 +178,28 @@
     <t>Pending</t>
   </si>
   <si>
+    <t>jason.t@tutors.com</t>
+  </si>
+  <si>
+    <t>david.k@tutors.com</t>
+  </si>
+  <si>
+    <t>nurul.h@tutors.com</t>
+  </si>
+  <si>
+    <t>marcus.c@tutors.com</t>
+  </si>
+  <si>
+    <t>priya.n@tutors.com</t>
+  </si>
+  <si>
+    <t>li.mei@tutors.com</t>
+  </si>
+  <si>
+    <t>sarah.l@tutors.com</t>
+  </si>
+  <si>
     <t>ahmad.r@tutors.com</t>
-  </si>
-  <si>
-    <t>priya.n@tutors.com</t>
-  </si>
-  <si>
-    <t>jason.t@tutors.com</t>
-  </si>
-  <si>
-    <t>david.k@tutors.com</t>
-  </si>
-  <si>
-    <t>nurul.h@tutors.com</t>
-  </si>
-  <si>
-    <t>marcus.c@tutors.com</t>
-  </si>
-  <si>
-    <t>li.mei@tutors.com</t>
-  </si>
-  <si>
-    <t>sarah.l@tutors.com</t>
   </si>
   <si>
     <t>Assignment ID</t>
@@ -603,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -619,31 +610,31 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -651,28 +642,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F2" s="1">
-        <v>55.0000</v>
+        <v>60.0000</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
         <v>54</v>
-      </c>
-      <c r="I2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -680,28 +671,25 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F3" s="1">
-        <v>45.0000</v>
+        <v>50.0000</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H3" t="s">
-        <v>54</v>
-      </c>
-      <c r="I3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -709,28 +697,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F4" s="1">
-        <v>60.0000</v>
+        <v>70.0000</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -738,25 +726,25 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F5" s="1">
         <v>50.0000</v>
       </c>
       <c r="G5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H5" t="s">
-        <v>54</v>
+        <v>51</v>
+      </c>
+      <c r="I5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -764,25 +752,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F6" s="1">
-        <v>55.0000</v>
+        <v>45.0000</v>
       </c>
       <c r="G6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I6" t="s">
         <v>57</v>
@@ -793,28 +781,28 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1">
-        <v>70.0000</v>
+        <v>45.0000</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -822,25 +810,28 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F8" s="1">
-        <v>50.0000</v>
+        <v>55.0000</v>
       </c>
       <c r="G8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -848,28 +839,28 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F9" s="1">
-        <v>45.0000</v>
+        <v>60.0000</v>
       </c>
       <c r="G9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" t="s">
         <v>54</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -877,28 +868,28 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F10" s="1">
         <v>45.0000</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -906,115 +897,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="D11" t="s">
-        <v>35</v>
-      </c>
       <c r="E11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F11" s="1">
         <v>55.0000</v>
       </c>
       <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
         <v>51</v>
       </c>
-      <c r="H11" t="s">
-        <v>54</v>
-      </c>
       <c r="I11" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="1">
-        <v>60.0000</v>
-      </c>
-      <c r="G12" t="s">
-        <v>52</v>
-      </c>
-      <c r="H12" t="s">
-        <v>56</v>
-      </c>
-      <c r="I12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="1">
-        <v>45.0000</v>
-      </c>
-      <c r="G13" t="s">
-        <v>53</v>
-      </c>
-      <c r="H13" t="s">
-        <v>54</v>
-      </c>
-      <c r="I13" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
-      </c>
-      <c r="E14" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" s="1">
-        <v>55.0000</v>
-      </c>
-      <c r="G14" t="s">
-        <v>44</v>
-      </c>
-      <c r="H14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>